<commit_message>
Verify and tighten analysis: fix Group 70 share, make the extra-fields check reproducible, derive text from data, add tests
</commit_message>
<xml_diff>
--- a/Incident_Routing_Impact_Model.xlsx
+++ b/Incident_Routing_Impact_Model.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\parul\Downloads\project3-incident-routing\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{89BF956B-F076-4008-8A7D-067B9B250904}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9F3D2E03-AD6C-44E4-8323-BB9FFD5FB55E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -65,7 +65,7 @@
     <t>incidents</t>
   </si>
   <si>
-    <t>[DATA] Average of Mar, Apr and May 2016 (350, 359, 356)</t>
+    <t>[DATA] Average of the three core months (350, 359, 356)</t>
   </si>
   <si>
     <t>First-time-right gain from the rule</t>

</xml_diff>